<commit_message>
chore: set row 10 demo access to 'None required (open local/Docker service)'
</commit_message>
<xml_diff>
--- a/Assessment4_Tharun_S.xlsx
+++ b/Assessment4_Tharun_S.xlsx
@@ -559,7 +559,7 @@
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
   <dimension ref="A1:C22"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="6" customWidth="1" style="12" min="1" max="1"/>
     <col width="96" customWidth="1" style="12" min="2" max="2"/>
@@ -761,7 +761,7 @@
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
   <dimension ref="A1:B18"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="34" customWidth="1" style="12" min="1" max="1"/>
     <col width="70" customWidth="1" style="12" min="2" max="2"/>
@@ -849,7 +849,11 @@
           <t>Live demo access token or login (if protected)</t>
         </is>
       </c>
-      <c r="B10" s="24" t="n"/>
+      <c r="B10" s="24" t="inlineStr">
+        <is>
+          <t>None required (open local/Docker service, no login required)</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="19.5" customHeight="1" s="13">
       <c r="A11" s="19" t="inlineStr">
@@ -961,7 +965,7 @@
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
   <dimension ref="A1:E14"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="5" customWidth="1" style="12" min="1" max="1"/>
     <col width="60" customWidth="1" style="12" min="2" max="2"/>
@@ -1304,7 +1308,7 @@
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
   <dimension ref="A1:E19"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="14" customWidth="1" style="12" min="1" max="1"/>
     <col width="62" customWidth="1" style="12" min="2" max="2"/>
@@ -1734,7 +1738,7 @@
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
   <dimension ref="A1:D15"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="30" customWidth="1" style="12" min="1" max="1"/>
     <col width="58" customWidth="1" style="12" min="2" max="2"/>
@@ -2039,7 +2043,7 @@
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
   <dimension ref="A1:E10"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="28" customWidth="1" style="12" min="1" max="1"/>
     <col width="50" customWidth="1" style="12" min="2" max="2"/>
@@ -2277,7 +2281,7 @@
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
   <dimension ref="A1:E11"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="5" customWidth="1" style="12" min="1" max="1"/>
     <col width="52" customWidth="1" style="12" min="2" max="2"/>
@@ -2534,7 +2538,7 @@
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
   <dimension ref="A1:B13"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="80" customWidth="1" style="12" min="1" max="1"/>
     <col width="14" customWidth="1" style="12" min="2" max="2"/>

</xml_diff>

<commit_message>
chore: add private github repository url to submission workbooks
</commit_message>
<xml_diff>
--- a/Assessment4_Tharun_S.xlsx
+++ b/Assessment4_Tharun_S.xlsx
@@ -873,7 +873,11 @@
           <t>Repository URL (private, reviewer invited)</t>
         </is>
       </c>
-      <c r="B12" s="24" t="n"/>
+      <c r="B12" s="24" t="inlineStr">
+        <is>
+          <t>https://github.com/Tectonic-s/incubrix-2026-ps4</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="19.5" customHeight="1" s="13">
       <c r="A13" s="19" t="inlineStr">

</xml_diff>